<commit_message>
feat(aposta-final): confirmação persistente da aposta salva
Antes o usuário só via um toast temporário após salvar e tinha que
inferir pelo selectbox que sua aposta estava registrada. Agora, no
topo da tela, aparece um banner verde resumindo a aposta atual
(campeão, vice, 3º, 4º) + quando foi atualizada. Se ainda não tem
aposta e a janela está aberta, banner azul orientando o próximo
passo.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pg.xlsx
+++ b/Pg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nexaiqbr-my.sharepoint.com/personal/charles_eduardo_nexaiq_com_br/Documents/NEXA/Bolao_Copa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0B6B10D-F7A5-4650-A42A-18C53DC8DD8F}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C76558E-255F-4D6A-B970-41170C3E6A93}"/>
   <bookViews>
-    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{832815FD-8D2E-45E2-9493-0C8D289D034C}"/>
+    <workbookView xWindow="2715" yWindow="0" windowWidth="21600" windowHeight="15585" xr2:uid="{832815FD-8D2E-45E2-9493-0C8D289D034C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="71">
   <si>
     <t>NOME</t>
   </si>
@@ -171,6 +171,87 @@
   </si>
   <si>
     <t>ROG</t>
+  </si>
+  <si>
+    <t>Rodrigo Nunes De Souza</t>
+  </si>
+  <si>
+    <t>Erico Castro</t>
+  </si>
+  <si>
+    <t>Paulo Rossi</t>
+  </si>
+  <si>
+    <t>Marcelo Pons Terruel</t>
+  </si>
+  <si>
+    <t>Diego Gabriel</t>
+  </si>
+  <si>
+    <t>Gabriel</t>
+  </si>
+  <si>
+    <t>Erico</t>
+  </si>
+  <si>
+    <t>Paulinho</t>
+  </si>
+  <si>
+    <t>Marcelo</t>
+  </si>
+  <si>
+    <t>Dieguinho</t>
+  </si>
+  <si>
+    <t>Russo</t>
+  </si>
+  <si>
+    <t>CUNHADO</t>
+  </si>
+  <si>
+    <t>Rodrigo 8</t>
+  </si>
+  <si>
+    <t>NAMO IZA</t>
+  </si>
+  <si>
+    <t>PAULO</t>
+  </si>
+  <si>
+    <t>1º</t>
+  </si>
+  <si>
+    <t>2º</t>
+  </si>
+  <si>
+    <t>3º</t>
+  </si>
+  <si>
+    <t>ALIEKSIEI MARTINS</t>
+  </si>
+  <si>
+    <t>ali</t>
+  </si>
+  <si>
+    <t>ANDERSON RIBEIRO DA SILVA</t>
+  </si>
+  <si>
+    <t>Anderson</t>
+  </si>
+  <si>
+    <t>Felippe Rossello</t>
+  </si>
+  <si>
+    <t>FehRoss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilian </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heitor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arthur </t>
   </si>
 </sst>
 </file>
@@ -227,11 +308,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -248,9 +330,16 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
     <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -264,6 +353,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -583,17 +676,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D625A835-F11C-41EC-844F-44F1F20CD40A}">
-  <dimension ref="A1:I112"/>
+  <dimension ref="A1:Q112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
     <col min="4" max="5" width="9.140625" style="1"/>
-    <col min="7" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -619,7 +713,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -637,18 +731,18 @@
       </c>
       <c r="G2" s="1">
         <f>COUNTA(A2:A1048576)</f>
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="H2" s="5">
         <f>SUMIFS(E:E,D:D,"PG")</f>
-        <v>450</v>
+        <v>720</v>
       </c>
       <c r="I2" s="5">
         <f>SUM(E2:E1048576)</f>
-        <v>510</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>33</v>
       </c>
@@ -665,7 +759,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
@@ -682,7 +776,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -699,7 +793,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -716,7 +810,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
@@ -726,11 +820,41 @@
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="D7" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="E7" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="O7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
@@ -746,8 +870,44 @@
       <c r="E8" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G8" s="5">
+        <f>$I$2*G9</f>
+        <v>609</v>
+      </c>
+      <c r="H8" s="5">
+        <f t="shared" ref="H8:I8" si="0">$I$2*H9</f>
+        <v>174</v>
+      </c>
+      <c r="I8" s="5">
+        <f t="shared" si="0"/>
+        <v>87</v>
+      </c>
+      <c r="K8" s="5">
+        <f>$I$2*K9</f>
+        <v>522</v>
+      </c>
+      <c r="L8" s="5">
+        <f t="shared" ref="L8" si="1">$I$2*L9</f>
+        <v>261</v>
+      </c>
+      <c r="M8" s="5">
+        <f t="shared" ref="M8" si="2">$I$2*M9</f>
+        <v>87</v>
+      </c>
+      <c r="O8" s="5">
+        <f>$I$2*O9</f>
+        <v>522</v>
+      </c>
+      <c r="P8" s="5">
+        <f t="shared" ref="P8" si="3">$I$2*P9</f>
+        <v>217.5</v>
+      </c>
+      <c r="Q8" s="5">
+        <f t="shared" ref="Q8" si="4">$I$2*Q9</f>
+        <v>130.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
@@ -757,11 +917,41 @@
       <c r="C9" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="D9" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="E9" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G9" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="H9" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="I9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="K9" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="L9" s="7">
+        <v>0.3</v>
+      </c>
+      <c r="M9" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="O9" s="7">
+        <v>0.6</v>
+      </c>
+      <c r="P9" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="Q9" s="7">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
@@ -778,7 +968,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
@@ -795,7 +985,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
@@ -812,7 +1002,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
@@ -829,7 +1019,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
@@ -846,7 +1036,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
@@ -863,7 +1053,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
@@ -915,76 +1105,193 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="E19" s="2"/>
+      <c r="A19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="E20" s="2"/>
+      <c r="A20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="E22" s="2"/>
+      <c r="A22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="E23" s="2"/>
+      <c r="A23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="E24" s="2"/>
+      <c r="A24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="E25" s="2"/>
+      <c r="A25" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="E26" s="2"/>
+      <c r="A26" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="E27" s="2"/>
+      <c r="A27" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="E28" s="2"/>
+      <c r="A28" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="E29" s="2"/>
+      <c r="A29" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="E30" s="2"/>
+      <c r="A30" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>

</xml_diff>

<commit_message>
feat(aposta-final): revela apostas de todos após a trava
Depois de 11/06 15:55 BRT (quando aposta_aberta retorna False),
aparece uma tabela nova "📋 Apostas Finais de todos os participantes"
listando apelido, nome, campeão, vice, 3º, 4º e pontos de cada um.
Mesma filosofia da Tela da Partida: palpite alheio só aparece
depois que ninguém pode mais mexer.

aposta_service.listar_apostas_completas: busca apostas com os 4 campos
preenchidos, junta com Usuario e Selecao em queries em batch (IN(...))
para evitar N+1, e ordena por pontos desc -> apelido.

Coluna "Pontos" só aparece quando alguém já tem ponto > 0
(antes do fim da Copa fica escondida).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pg.xlsx
+++ b/Pg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nexaiqbr-my.sharepoint.com/personal/charles_eduardo_nexaiq_com_br/Documents/NEXA/Bolao_Copa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C76558E-255F-4D6A-B970-41170C3E6A93}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1590CBD8-C838-4C31-B4DB-4551EE1AE288}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="0" windowWidth="21600" windowHeight="15585" xr2:uid="{832815FD-8D2E-45E2-9493-0C8D289D034C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{832815FD-8D2E-45E2-9493-0C8D289D034C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="76">
   <si>
     <t>NOME</t>
   </si>
@@ -252,6 +252,21 @@
   </si>
   <si>
     <t xml:space="preserve">Arthur </t>
+  </si>
+  <si>
+    <t>Feliphi</t>
+  </si>
+  <si>
+    <t>Lacerda</t>
+  </si>
+  <si>
+    <t>Arthur</t>
+  </si>
+  <si>
+    <t>Heitor</t>
+  </si>
+  <si>
+    <t>Lilian</t>
   </si>
 </sst>
 </file>
@@ -731,15 +746,15 @@
       </c>
       <c r="G2" s="1">
         <f>COUNTA(A2:A1048576)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H2" s="5">
         <f>SUMIFS(E:E,D:D,"PG")</f>
-        <v>720</v>
+        <v>870</v>
       </c>
       <c r="I2" s="5">
         <f>SUM(E2:E1048576)</f>
-        <v>870</v>
+        <v>900</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -872,39 +887,39 @@
       </c>
       <c r="G8" s="5">
         <f>$I$2*G9</f>
-        <v>609</v>
+        <v>630</v>
       </c>
       <c r="H8" s="5">
         <f t="shared" ref="H8:I8" si="0">$I$2*H9</f>
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="I8" s="5">
         <f t="shared" si="0"/>
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="K8" s="5">
         <f>$I$2*K9</f>
-        <v>522</v>
+        <v>540</v>
       </c>
       <c r="L8" s="5">
         <f t="shared" ref="L8" si="1">$I$2*L9</f>
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="M8" s="5">
         <f t="shared" ref="M8" si="2">$I$2*M9</f>
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="O8" s="5">
         <f>$I$2*O9</f>
-        <v>522</v>
+        <v>540</v>
       </c>
       <c r="P8" s="5">
         <f t="shared" ref="P8" si="3">$I$2*P9</f>
-        <v>217.5</v>
+        <v>225</v>
       </c>
       <c r="Q8" s="5">
         <f t="shared" ref="Q8" si="4">$I$2*Q9</f>
-        <v>130.5</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
@@ -1165,6 +1180,9 @@
       <c r="C22" s="3" t="s">
         <v>21</v>
       </c>
+      <c r="D22" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="E22" s="2">
         <v>30</v>
       </c>
@@ -1256,10 +1274,13 @@
         <v>68</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>21</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="E28" s="2">
         <v>30</v>
@@ -1270,10 +1291,13 @@
         <v>69</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>21</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="E29" s="2">
         <v>30</v>
@@ -1284,20 +1308,34 @@
         <v>70</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>21</v>
       </c>
+      <c r="D30" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="E30" s="2">
         <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="E31" s="2"/>
+      <c r="A31" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31" s="2">
+        <v>30</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>

</xml_diff>

<commit_message>
ui: default inteligente da partida em "Tela da Partida" e Admin -> Resultados
helpers.indice_partida_default ordena por: 1) em_andamento, 2) próxima a
começar, 3) última. Tela da Partida e Admin -> Resultados agora caem
direto no jogo "do momento" em vez do primeiro de toda a Copa. Os
filtros (data e grupos/fase) seguem funcionando por cima.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pg.xlsx
+++ b/Pg.xlsx
@@ -8,13 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nexaiqbr-my.sharepoint.com/personal/charles_eduardo_nexaiq_com_br/Documents/NEXA/Bolao_Copa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="111" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1590CBD8-C838-4C31-B4DB-4551EE1AE288}"/>
+  <xr:revisionPtr revIDLastSave="119" documentId="8_{9DC803D6-6F12-4051-A5B7-BF4F5480704B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0924EC5-3FBD-4B38-AE71-1AFDD9C3F697}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{832815FD-8D2E-45E2-9493-0C8D289D034C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$F$31</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="77">
   <si>
     <t>NOME</t>
   </si>
@@ -267,6 +273,9 @@
   </si>
   <si>
     <t>Lilian</t>
+  </si>
+  <si>
+    <t>#</t>
   </si>
 </sst>
 </file>
@@ -368,6 +377,153 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="2026-06-11T19-01_export"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="A1" t="str">
+            <v>Apelido</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>ali</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3" t="str">
+            <v>Aninha</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>Arthur</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>Churros</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6" t="str">
+            <v>corinthians</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7" t="str">
+            <v>Delbuque</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8" t="str">
+            <v>Dieguinho</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9" t="str">
+            <v>dxjao</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10" t="str">
+            <v>Erico</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="A11" t="str">
+            <v>FehRoss</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="A12" t="str">
+            <v>Heitor</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="A13" t="str">
+            <v>iarossi</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="A14" t="str">
+            <v>Iza</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="A15" t="str">
+            <v>jerangel</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="A16" t="str">
+            <v>Kaue</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="A17" t="str">
+            <v>Lacerda</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="A18" t="str">
+            <v>Lilian</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="A19" t="str">
+            <v>Marcelo</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="A20" t="str">
+            <v>Nariz</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="A21" t="str">
+            <v>Paulinho</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="A22" t="str">
+            <v>Ramonzito</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="A23" t="str">
+            <v>Renato</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="A24" t="str">
+            <v>Rodrigo 8</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="A25" t="str">
+            <v>Ronaldo</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="A26" t="str">
+            <v>Russo</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -691,18 +847,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D625A835-F11C-41EC-844F-44F1F20CD40A}">
-  <dimension ref="A1:Q112"/>
+  <dimension ref="A1:R112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="9.140625" style="1"/>
-    <col min="7" max="7" width="11.28515625" customWidth="1"/>
-    <col min="8" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="1" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" style="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -710,1120 +866,1328 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="3" t="str">
+        <f>VLOOKUP(B2,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Nariz</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="2">
-        <v>30</v>
-      </c>
-      <c r="G2" s="1">
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2">
+        <v>30</v>
+      </c>
+      <c r="H2" s="1">
         <f>COUNTA(A2:A1048576)</f>
         <v>30</v>
       </c>
-      <c r="H2" s="5">
-        <f>SUMIFS(E:E,D:D,"PG")</f>
-        <v>870</v>
-      </c>
       <c r="I2" s="5">
-        <f>SUM(E2:E1048576)</f>
+        <f>SUMIFS(F:F,E:E,"PG")</f>
         <v>900</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="J2" s="5">
+        <f>SUM(F2:F1048576)</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="3" t="str">
+        <f>VLOOKUP(B3,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Kaue</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="3" t="str">
+        <f>VLOOKUP(B4,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Churros</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="3" t="str">
+        <f>VLOOKUP(B5,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Renato</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="3" t="str">
+        <f>VLOOKUP(B6,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Delbuque</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="3" t="str">
+        <f>VLOOKUP(B7,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Iza</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" s="2">
-        <v>30</v>
-      </c>
-      <c r="G7" s="6" t="s">
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="2">
+        <v>30</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="I7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="L7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="M7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="N7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="O7" s="6" t="s">
+      <c r="P7" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="P7" s="4" t="s">
+      <c r="Q7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="Q7" s="4" t="s">
+      <c r="R7" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="3" t="str">
+        <f>VLOOKUP(B8,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Ramonzito</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="2">
-        <v>30</v>
-      </c>
-      <c r="G8" s="5">
-        <f>$I$2*G9</f>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2">
+        <v>30</v>
+      </c>
+      <c r="H8" s="5">
+        <f>$J$2*H9</f>
         <v>630</v>
       </c>
-      <c r="H8" s="5">
-        <f t="shared" ref="H8:I8" si="0">$I$2*H9</f>
+      <c r="I8" s="5">
+        <f t="shared" ref="I8:J8" si="0">$J$2*I9</f>
         <v>180</v>
       </c>
-      <c r="I8" s="5">
+      <c r="J8" s="5">
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="K8" s="5">
-        <f>$I$2*K9</f>
+      <c r="L8" s="5">
+        <f>$J$2*L9</f>
         <v>540</v>
       </c>
-      <c r="L8" s="5">
-        <f t="shared" ref="L8" si="1">$I$2*L9</f>
+      <c r="M8" s="5">
+        <f t="shared" ref="M8" si="1">$J$2*M9</f>
         <v>270</v>
       </c>
-      <c r="M8" s="5">
-        <f t="shared" ref="M8" si="2">$I$2*M9</f>
+      <c r="N8" s="5">
+        <f t="shared" ref="N8" si="2">$J$2*N9</f>
         <v>90</v>
       </c>
-      <c r="O8" s="5">
-        <f>$I$2*O9</f>
+      <c r="P8" s="5">
+        <f>$J$2*P9</f>
         <v>540</v>
       </c>
-      <c r="P8" s="5">
-        <f t="shared" ref="P8" si="3">$I$2*P9</f>
+      <c r="Q8" s="5">
+        <f t="shared" ref="Q8" si="3">$J$2*Q9</f>
         <v>225</v>
       </c>
-      <c r="Q8" s="5">
-        <f t="shared" ref="Q8" si="4">$I$2*Q9</f>
+      <c r="R8" s="5">
+        <f t="shared" ref="R8" si="4">$J$2*R9</f>
         <v>135</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="3" t="str">
+        <f>VLOOKUP(B9,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>jerangel</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="2">
-        <v>30</v>
-      </c>
-      <c r="G9" s="7">
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="2">
+        <v>30</v>
+      </c>
+      <c r="H9" s="7">
         <v>0.7</v>
       </c>
-      <c r="H9" s="7">
+      <c r="I9" s="7">
         <v>0.2</v>
       </c>
-      <c r="I9" s="7">
+      <c r="J9" s="7">
         <v>0.1</v>
       </c>
-      <c r="K9" s="7">
+      <c r="L9" s="7">
         <v>0.6</v>
       </c>
-      <c r="L9" s="7">
+      <c r="M9" s="7">
         <v>0.3</v>
       </c>
-      <c r="M9" s="7">
+      <c r="N9" s="7">
         <v>0.1</v>
       </c>
-      <c r="O9" s="7">
+      <c r="P9" s="7">
         <v>0.6</v>
       </c>
-      <c r="P9" s="7">
+      <c r="Q9" s="7">
         <v>0.25</v>
       </c>
-      <c r="Q9" s="7">
+      <c r="R9" s="7">
         <v>0.15</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="3" t="e">
+        <f>VLOOKUP(B10,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="3" t="str">
+        <f>VLOOKUP(B11,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Aninha</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F11" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="3" t="str">
+        <f>VLOOKUP(B12,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Ronaldo</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F12" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="3" t="str">
+        <f>VLOOKUP(B13,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>dxjao</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="3" t="str">
+        <f>VLOOKUP(B14,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>corinthians</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E14" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="3" t="e">
+        <f>VLOOKUP(B15,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="3" t="str">
+        <f>VLOOKUP(B16,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>iarossi</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="3" t="e">
+        <f>VLOOKUP(B17,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E17" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E17" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="3" t="e">
+        <f>VLOOKUP(B18,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E18" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="3" t="str">
+        <f>VLOOKUP(B19,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Rodrigo 8</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E19" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F19" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>45</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="3" t="str">
+        <f>VLOOKUP(B20,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Erico</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E20" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="3" t="str">
+        <f>VLOOKUP(B21,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Paulinho</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E21" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E21" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>47</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="3" t="str">
+        <f>VLOOKUP(B22,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Marcelo</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E22" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F22" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>48</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="3" t="str">
+        <f>VLOOKUP(B23,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Dieguinho</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E23" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F23" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="3" t="str">
+        <f>VLOOKUP(B24,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Russo</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F24" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="3" t="str">
+        <f>VLOOKUP(B25,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>ali</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E25" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F25" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>64</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="3" t="e">
+        <f>VLOOKUP(B26,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E26" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F26" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>66</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="3" t="str">
+        <f>VLOOKUP(B27,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>FehRoss</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D27" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E27" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F27" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>68</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="3" t="str">
+        <f>VLOOKUP(B28,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Lilian</v>
+      </c>
+      <c r="D28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E28" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F28" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>69</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="3" t="str">
+        <f>VLOOKUP(B29,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Heitor</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E29" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F29" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>70</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="3" t="s">
+      <c r="C30" s="3" t="str">
+        <f>VLOOKUP(B30,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Arthur</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F30" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>71</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="3" t="str">
+        <f>VLOOKUP(B31,'[1]2026-06-11T19-01_export'!$A:$A,1,0)</f>
+        <v>Lacerda</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E31" s="2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F31" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
-      <c r="E32" s="2"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D32" s="3"/>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
-      <c r="E33" s="2"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D33" s="3"/>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
-      <c r="E34" s="2"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D34" s="3"/>
+      <c r="F34" s="2"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
-      <c r="E35" s="2"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D35" s="3"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
-      <c r="E36" s="2"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D36" s="3"/>
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
-      <c r="E37" s="2"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D37" s="3"/>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="E38" s="2"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D38" s="3"/>
+      <c r="F38" s="2"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
-      <c r="E39" s="2"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D39" s="3"/>
+      <c r="F39" s="2"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="E40" s="2"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D40" s="3"/>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="E41" s="2"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D41" s="3"/>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
-      <c r="E42" s="2"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D42" s="3"/>
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
-      <c r="E43" s="2"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D43" s="3"/>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
-      <c r="E44" s="2"/>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D44" s="3"/>
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D45" s="3"/>
+      <c r="F45" s="2"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
-      <c r="E46" s="2"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D46" s="3"/>
+      <c r="F46" s="2"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
-      <c r="E47" s="2"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D47" s="3"/>
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
-      <c r="E48" s="2"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D48" s="3"/>
+      <c r="F48" s="2"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
-      <c r="E49" s="2"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D49" s="3"/>
+      <c r="F49" s="2"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
-      <c r="E50" s="2"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D50" s="3"/>
+      <c r="F50" s="2"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
-      <c r="E51" s="2"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D51" s="3"/>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
-      <c r="E52" s="2"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D52" s="3"/>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
-      <c r="E53" s="2"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D53" s="3"/>
+      <c r="F53" s="2"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
-      <c r="E54" s="2"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D54" s="3"/>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
-      <c r="E55" s="2"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D55" s="3"/>
+      <c r="F55" s="2"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
-      <c r="E56" s="2"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D56" s="3"/>
+      <c r="F56" s="2"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
-      <c r="E57" s="2"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D57" s="3"/>
+      <c r="F57" s="2"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
-      <c r="E58" s="2"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D58" s="3"/>
+      <c r="F58" s="2"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
-      <c r="E59" s="2"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D59" s="3"/>
+      <c r="F59" s="2"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
-      <c r="E60" s="2"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D60" s="3"/>
+      <c r="F60" s="2"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
-      <c r="E61" s="2"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D61" s="3"/>
+      <c r="F61" s="2"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
-      <c r="E62" s="2"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D62" s="3"/>
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
-      <c r="E63" s="2"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D63" s="3"/>
+      <c r="F63" s="2"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
-      <c r="E64" s="2"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D64" s="3"/>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
-      <c r="E65" s="2"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D65" s="3"/>
+      <c r="F65" s="2"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
-      <c r="E66" s="2"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D66" s="3"/>
+      <c r="F66" s="2"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
-      <c r="E67" s="2"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D67" s="3"/>
+      <c r="F67" s="2"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
-      <c r="E68" s="2"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D68" s="3"/>
+      <c r="F68" s="2"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
-      <c r="E69" s="2"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D69" s="3"/>
+      <c r="F69" s="2"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
-      <c r="E70" s="2"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D70" s="3"/>
+      <c r="F70" s="2"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
-      <c r="E71" s="2"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D71" s="3"/>
+      <c r="F71" s="2"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
-      <c r="E72" s="2"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D72" s="3"/>
+      <c r="F72" s="2"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
-      <c r="E73" s="2"/>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D73" s="3"/>
+      <c r="F73" s="2"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
-      <c r="E74" s="2"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D74" s="3"/>
+      <c r="F74" s="2"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
-      <c r="E75" s="2"/>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D75" s="3"/>
+      <c r="F75" s="2"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
-      <c r="E76" s="2"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D76" s="3"/>
+      <c r="F76" s="2"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
-      <c r="E77" s="2"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D77" s="3"/>
+      <c r="F77" s="2"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
-      <c r="E78" s="2"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D78" s="3"/>
+      <c r="F78" s="2"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
-      <c r="E79" s="2"/>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D79" s="3"/>
+      <c r="F79" s="2"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
-      <c r="E80" s="2"/>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D80" s="3"/>
+      <c r="F80" s="2"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
-      <c r="E81" s="2"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D81" s="3"/>
+      <c r="F81" s="2"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
-      <c r="E82" s="2"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D82" s="3"/>
+      <c r="F82" s="2"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
-      <c r="E83" s="2"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D83" s="3"/>
+      <c r="F83" s="2"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
-      <c r="E84" s="2"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D84" s="3"/>
+      <c r="F84" s="2"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
-      <c r="E85" s="2"/>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D85" s="3"/>
+      <c r="F85" s="2"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
-      <c r="E86" s="2"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D86" s="3"/>
+      <c r="F86" s="2"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
-      <c r="E87" s="2"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D87" s="3"/>
+      <c r="F87" s="2"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
-      <c r="E88" s="2"/>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D88" s="3"/>
+      <c r="F88" s="2"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
-      <c r="E89" s="2"/>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D89" s="3"/>
+      <c r="F89" s="2"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
-      <c r="E90" s="2"/>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D90" s="3"/>
+      <c r="F90" s="2"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
-      <c r="E91" s="2"/>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D91" s="3"/>
+      <c r="F91" s="2"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
-      <c r="E92" s="2"/>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D92" s="3"/>
+      <c r="F92" s="2"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
-      <c r="E93" s="2"/>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D93" s="3"/>
+      <c r="F93" s="2"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
-      <c r="E94" s="2"/>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D94" s="3"/>
+      <c r="F94" s="2"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
-      <c r="E95" s="2"/>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D95" s="3"/>
+      <c r="F95" s="2"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
-      <c r="E96" s="2"/>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D96" s="3"/>
+      <c r="F96" s="2"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
-      <c r="E97" s="2"/>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D97" s="3"/>
+      <c r="F97" s="2"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
-      <c r="E98" s="2"/>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D98" s="3"/>
+      <c r="F98" s="2"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
-      <c r="E99" s="2"/>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D99" s="3"/>
+      <c r="F99" s="2"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
-      <c r="E100" s="2"/>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D100" s="3"/>
+      <c r="F100" s="2"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
-      <c r="E101" s="2"/>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D101" s="3"/>
+      <c r="F101" s="2"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
-      <c r="E102" s="2"/>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D102" s="3"/>
+      <c r="F102" s="2"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
-      <c r="E103" s="2"/>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D103" s="3"/>
+      <c r="F103" s="2"/>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
-      <c r="E104" s="2"/>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D104" s="3"/>
+      <c r="F104" s="2"/>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
-      <c r="E105" s="2"/>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D105" s="3"/>
+      <c r="F105" s="2"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
-      <c r="E106" s="2"/>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D106" s="3"/>
+      <c r="F106" s="2"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
-      <c r="E107" s="2"/>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D107" s="3"/>
+      <c r="F107" s="2"/>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
-      <c r="E108" s="2"/>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D108" s="3"/>
+      <c r="F108" s="2"/>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
-      <c r="E109" s="2"/>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D109" s="3"/>
+      <c r="F109" s="2"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
-      <c r="E110" s="2"/>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D110" s="3"/>
+      <c r="F110" s="2"/>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
-      <c r="E111" s="2"/>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D111" s="3"/>
+      <c r="F111" s="2"/>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
-      <c r="E112" s="2"/>
+      <c r="D112" s="3"/>
+      <c r="F112" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F31" xr:uid="{D625A835-F11C-41EC-844F-44F1F20CD40A}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>